<commit_message>
update diapo et figures
</commit_message>
<xml_diff>
--- a/figures/dataset_CLV.xlsx
+++ b/figures/dataset_CLV.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\g.martet\Documents\Agrostat Dijon\figures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D2EF3F80-E526-462F-8DC4-9FC840C5837E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6FEAA8D-1D0E-42B3-8A2F-479A6D4CC779}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E12FFB58-BF93-4D82-9450-4001AA5E4D95}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{E12FFB58-BF93-4D82-9450-4001AA5E4D95}"/>
   </bookViews>
   <sheets>
-    <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
+    <sheet name="CLV" sheetId="1" r:id="rId1"/>
+    <sheet name="Feuil1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="53">
   <si>
     <t>Région</t>
   </si>
@@ -76,13 +77,373 @@
   </si>
   <si>
     <t>cluster 2</t>
+  </si>
+  <si>
+    <t>Block</t>
+  </si>
+  <si>
+    <t>Variable name</t>
+  </si>
+  <si>
+    <t>fPC1 interpretation</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>AMR_ville_FQ_R</t>
+  </si>
+  <si>
+    <t>AMC</t>
+  </si>
+  <si>
+    <t>log_AMC_ville_FQ</t>
+  </si>
+  <si>
+    <t>log_AMC_ES_FQ</t>
+  </si>
+  <si>
+    <t>Humans</t>
+  </si>
+  <si>
+    <t>medecin_hab</t>
+  </si>
+  <si>
+    <t>Animals</t>
+  </si>
+  <si>
+    <t>veto_by_AC</t>
+  </si>
+  <si>
+    <t>log_UGB_density_livestock_tot</t>
+  </si>
+  <si>
+    <t>AMR_animaux_compagnie_FQ_R</t>
+  </si>
+  <si>
+    <t>AMR_animaux_production_FQ_R</t>
+  </si>
+  <si>
+    <t>Environment</t>
+  </si>
+  <si>
+    <t>air_PM25</t>
+  </si>
+  <si>
+    <t>dju_refroi</t>
+  </si>
+  <si>
+    <t>fPC1 % var</t>
+  </si>
+  <si>
+    <t>98.9%</t>
+  </si>
+  <si>
+    <t>93.1%</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>EQI_st</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (European quality of government index)</t>
+    </r>
+  </si>
+  <si>
+    <t>81.3%</t>
+  </si>
+  <si>
+    <t>76.9%</t>
+  </si>
+  <si>
+    <t>92.4%</t>
+  </si>
+  <si>
+    <t>85.8%</t>
+  </si>
+  <si>
+    <t>91.1%</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Consumption of Fluoroquinolone in primary care setting over the time</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: PACA, Occitanie ↑ VS Bretagne, Pays de la Loire ↓</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Consumption of Fluoroquinolone in hospitals over the time</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Grand-Est, PACA, Occitanie ↑ VS Bretagne, Pays de la Loire ↓</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Citizens’ trust in the quality, impartiality, and reliability of public institutions over the time:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Bretagne ↑ VS PACA ↓</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Number of doctors per population over the time</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: PACA, IDF ↑ VS Normandie, Centre-Val de Loire, Hauts-de-France↓ </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Fluoroquinolone resistance in pets over the time</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: PACA, IDF ↑ VS Centre-Val de Loire ↓</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Number of vet per pet over the time</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Bretagne ↑ VS Hauts-de-France, Centre Val-de-loire ↓</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Livestock density over the time</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Bretagne ↑ VS IDF ↓</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Fluoroquinolone resistance in livestock over the time</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Occitanie ↑ VS all other regions ↓</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Proportion of fine particles measuring 2.5 micrometers over the time</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Hauts-de-France, IDF ↑ VS Bretagne, Nouvelle-Aquitaine ↓</t>
+    </r>
+  </si>
+  <si>
+    <t>97.4%</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Accumulated difference between daily outdoor temperatures and a reference temperature above which cooling is needed over the time</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: PACA, Occitanie ↑ VS Bretagne, Normandie ↓</t>
+    </r>
+  </si>
+  <si>
+    <t>92.8%</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Fluoroquinolone resistance in primary care setting over the time</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: PACA ↑ VS Centre-Val-de-Loire ↓</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -90,8 +451,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -113,6 +482,36 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFACC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8766D"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA3A500"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE76BF3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00BF7D"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -181,17 +580,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -207,11 +612,80 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -221,6 +695,11 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FF00BF7D"/>
+      <color rgb="FF00B0F6"/>
+      <color rgb="FFE76BF3"/>
+      <color rgb="FFA3A500"/>
+      <color rgb="FFF8766D"/>
       <color rgb="FFFFFACC"/>
       <color rgb="FF00AC8C"/>
     </mruColors>
@@ -534,251 +1013,251 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D27BBFA5-915D-4CED-936B-1A2746899247}">
   <dimension ref="A1:K13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="6" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="6" width="9.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A1" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="I1" s="1" t="s">
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="I1" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I2" s="5"/>
-      <c r="J2" s="11" t="s">
+      <c r="I2" s="4"/>
+      <c r="J2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="K2" s="12" t="s">
+      <c r="K2" s="6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="I3" s="2" t="s">
+      <c r="B3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="J3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="K3" s="4" t="s">
+      <c r="K3" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="I4" s="2" t="s">
+      <c r="B4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="J4" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="K4" s="4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+      <c r="J4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="I5" s="2" t="s">
+      <c r="B5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="I6" s="2" t="s">
+      <c r="J5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="I6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J6" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="J6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A8" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="5"/>
-      <c r="B9" s="6" t="s">
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A9" s="4"/>
+      <c r="B9" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="7"/>
-      <c r="D9" s="8" t="s">
+      <c r="C9" s="9"/>
+      <c r="D9" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="9"/>
-      <c r="F9" s="10"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+      <c r="E9" s="11"/>
+      <c r="F9" s="12"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="F10" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+      <c r="B11" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B12" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+      <c r="B12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F13" s="4" t="s">
+      <c r="B13" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F13" s="3" t="s">
         <v>9</v>
       </c>
     </row>
@@ -792,4 +1271,183 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C00E3398-53EF-4F84-88FD-DB80C001C280}">
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.81640625" style="13" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.54296875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="40.1796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D1" s="14" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" s="21" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="18"/>
+      <c r="B4" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" s="21" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="C5" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="22"/>
+      <c r="B6" s="26" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="27">
+        <v>0.99</v>
+      </c>
+      <c r="D6" s="25" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A7" s="28" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="30" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="31" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A8" s="28"/>
+      <c r="B8" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="30" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" s="31" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A9" s="28"/>
+      <c r="B9" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="32">
+        <v>1</v>
+      </c>
+      <c r="D9" s="31" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A10" s="28"/>
+      <c r="B10" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" s="31" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A11" s="33" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" s="34" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="35" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" s="36" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="68.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="33"/>
+      <c r="B12" s="34" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12" s="37" t="s">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="A7:A10"/>
+    <mergeCell ref="A11:A12"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>